<commit_message>
Updated the DashboardPage to wait for adminPanel button to be visible before it is clicked on and expanded the page on the BasePage
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\refilwem\PlaywrightProject\playright2026Project\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DB7D54-7D2F-4990-8967-2B9A07E5E4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49578EA-71C9-4274-9C98-7799272C85A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DACBAD44-249F-4121-AFC4-BA9015D5A569}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DACBAD44-249F-4121-AFC4-BA9015D5A569}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
     <t>status</t>
   </si>
   <si>
-    <t>testerref2026@ndosi.com</t>
-  </si>
-  <si>
     <t>Tester2026!</t>
   </si>
   <si>
@@ -78,6 +75,9 @@
   </si>
   <si>
     <t>Testing Academy Co</t>
+  </si>
+  <si>
+    <t>testerrm@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -124,8 +124,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -495,31 +495,31 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="1">
+        <v>46212</v>
+      </c>
+      <c r="G2" t="s">
         <v>10</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46212</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{C398700C-A601-4C01-9502-F2C8D95BE243}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{74D978BD-034F-4FF3-AE9A-C094209BC4FE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>